<commit_message>
pm pack: add Phase 2 — AWS cloud migration & scale to 5,000 users (E11 cloud platform, E12 scale/performance, E13 production integration & ops); 4 rebalanced sprints (7-10), 30 stories, 131 SP
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/regagg/planning/Regulatory_Aggregator_Roadmap.xlsx
+++ b/docs/regagg/planning/Regulatory_Aggregator_Roadmap.xlsx
@@ -14,8 +14,8 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Capacity!$A$1:$F$6</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Epics!$A$1:$C$11</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Roadmap!$A$1:$I$73</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Epics!$A$1:$C$14</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Roadmap!$A$1:$I$103</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="480">
   <si>
     <t xml:space="preserve">Story ID</t>
   </si>
@@ -866,6 +866,396 @@
     <t xml:space="preserve">Readiness review held; handover acknowledged</t>
   </si>
   <si>
+    <t xml:space="preserve">REG-801</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cloud Migration &amp; Data Platform (AWS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Infrastructure-as-code baseline for the aggregator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Codify the aggregator's AWS footprint (RDS access, S3 buckets/prefixes, ECR repo, ECS task definitions, EventBridge rules, IAM roles) as reviewable IaC in the platform's existing tooling, with per-environment parameters.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dev/staging/prod stacks deploy from code with no console steps; IAM follows least privilege; teardown/redeploy reproduces an identical environment; peer-reviewed and merged</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-802</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PostgreSQL migration &amp; schema deployment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deploy the reg_* schema into the existing production PostgreSQL (namespaced, no collisions with platform tables) and migrate the SQLite corpus index with full fidelity; establish forward migration tooling.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All 9 reg_* tables created via versioned migration; row counts and invariants match source exactly; one-current-per-doc enforced by partial unique index; rollback path documented; full test suite green against Postgres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-803</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S3 storage cutover for corpus and markdown projection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Switch the storage backend from local disk to S3 for the canonical corpus (raw/meta/versions/archive) and the agent-facing markdown projection, preserving the exact key layout the agent tools consume.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Existing ~6GB corpus migrated with checksum verification; ingestion writes to S3; projection paths unchanged for agent tools; archive immutability enforced via bucket policy/versioning; no local-disk dependency remains</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secrets and environment configuration management</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Move API keys, database credentials and per-environment settings into the platform's secrets manager/parameter store; remove file-based keys; document rotation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No credential exists in the repo or on disk; application resolves secrets at runtime per environment; key rotation performed without redeploy; rotation SOP documented</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Containerise collection workers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Package the collection pipeline as a container image (pinned dependencies, non-root, health check) published to the registry, runnable as a one-shot task.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Image builds reproducibly in CI; a task run performs a full regulator ingest against RDS+S3; image scanned for vulnerabilities with no criticals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-806</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cloud-scheduled daily and weekly ingestion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replace host cron with cloud scheduling: daily delta run and weekly deep run as scheduled container tasks, with concurrency guard, timeout, retry and failure notification.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daily/weekly schedules fire reliably; overlapping runs prevented; failures raise an alert; run history visible in the existing dashboard exactly as today</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-807</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cloud backup, retention and restore drill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adopt platform-native durability: RDS automated backups with point-in-time recovery, S3 versioning plus lifecycle tiering for archive, and a documented restore procedure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PITR verified by restoring to a scratch instance; S3 versioning protects against accidental deletion; lifecycle policy moves cold archive to cheaper tier; restore drill timed and documented against RPO/RTO targets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-808</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BA: data classification, residency and retention sign-off</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm classification of the corpus (public regulatory content plus internal metadata), residency requirements and retention obligations for the cloud footprint.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Classification recorded; residency constraints reflected in region/bucket choices; retention schedule agreed with compliance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PM-S7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PM: sprint ceremonies, cloud dependency management</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recurring PM allocation plus coordination with the platform team.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ceremonies held; cross-team dependencies tracked; sprint report issued</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-901</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Production Integration, Security &amp; Operations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Register reg_* tools on the production MCP server</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deploy the twelve reg_* tool definitions into the existing production MCP server so the production agent can call them, without forking platform code.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All twelve tools discoverable and callable in production; naming does not collide with existing platform tools; mutating tool (trigger run) gated by role; smoke test from the production agent passes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scale &amp; Performance (100 → 5,000 users)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eliminate per-row object-store reads on the read path</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove N+1 storage reads: persist document excerpts as a database column at ingest instead of reading each markdown file per listing row, and stop reading document bodies during search scoring.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corpus listing issues a single database query with zero object-store calls; excerpt backfilled for existing corpus and maintained at ingest; p95 listing latency under target with cold cache</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-903</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delegate content search to the platform search layer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point content retrieval at the platform's existing BM25/RAG index over the markdown projection, keeping the filter-then-rank contract; retire the interim in-process scorer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reg_search filters in SQL then ranks via the platform index; results and citations equivalent or better than interim ranker; latency budget met on the full corpus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-904</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horizontally scalable stateless read tier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run the dashboard/API tier as stateless replicas behind the platform load balancer with autoscaling, connection pooling to RDS, and graceful shutdown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service scales out and in under load with no session affinity; database connections bounded and pooled; rolling deploy causes no failed requests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Response caching for hot read endpoints</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cache coverage tree, facet counts and change-feed responses with short, explicit TTLs and invalidation on ingest completion.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repeat dashboard loads served from cache; cache invalidated within one minute of a completed run; cache hit ratio and staleness observable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-906</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SSO authentication and role-based access control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replace single-operator access with platform SSO and two roles: analyst (read) and operator (run, toggle, manual ingest); identity flows into the existing audit trail.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unauthenticated access refused; analysts cannot trigger runs or manual ingests; every mutating action recorded with the authenticated identity; access matrix matches the signed-off definition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-907</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per-tenant API keys, quotas and rate limiting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Issue scoped keys per team/agent with request quotas and rate limits so one consumer cannot degrade the service for 5,000 users.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keys scoped to reg_* tools; quota and rate limit enforced with clear error responses; usage attributable per key; limits configurable without redeploy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-908</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Queue-based parallel ingestion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Introduce a work queue between detection and fetch so multiple workers process documents concurrently, keeping the daily window comfortable as coverage depth grows, while preserving per-regulator politeness limits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full fleet run completes within the agreed window; per-domain rate limits still honoured; failures isolated per document; ordering-independent and idempotent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-909</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BA: role and access matrix definition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Define analyst/operator/administrator permissions across UI and tools and obtain security sign-off.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matrix signed off; mapped to implemented roles; exceptions documented</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PM-S8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PM: sprint ceremonies, integration coordination</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recurring PM allocation plus platform-team integration coordination.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ceremonies held; integration risks tracked; sprint report issued</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-1001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load and soak testing to 5,000 users</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Define SLOs and prove them: model realistic analyst and agent traffic, run peak-load and multi-hour soak tests including a concurrent ingestion window.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agreed SLOs documented; peak load sustained within latency budgets; soak shows no memory/connection leak; results reported with headroom analysis and breaking point identified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-1002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Performance tuning from load-test findings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address the bottlenecks the load test surfaces: query plans and indexes, pagination limits, payload sizes, and any remaining chatty calls.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each identified bottleneck has a measured before/after; SLOs met with agreed headroom; changes covered by regression tests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-1003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observability: metrics, logs and dashboards</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emit structured logs and service metrics (ingestion volume and errors, corpus freshness, tool latency and error rate, queue depth) into the platform's monitoring stack with an operations dashboard.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Golden signals visible per service; ingestion and corpus health tracked over time; logs correlatable by run and request identifier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-1004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alerting and operational runbooks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alert on the conditions that matter — failed or missed daily run, regulator staleness beyond threshold, integrity violation, elevated tool error rate — each with a runbook.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every alert has an owner, severity and runbook; alerts tested by injecting each condition; no alert without a documented response</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-1005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CI/CD pipeline with automated quality gates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automate build, test and deployment: full test suite and foundation gate on every change, image build and scan, staged deployment with rollback.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No manual deployment steps; pipeline blocks on failing tests or critical vulnerabilities; rollback exercised successfully at least once</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-1006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Security review and hardening</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Complete pre-production security work: TLS everywhere, no default credentials, least-privilege IAM and bucket policies, dependency and image scanning, remediation of review findings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Security review passed with no open high findings; default credentials eliminated; egress allow-list covers regulator domains; findings tracked to closure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-1007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost model and optimisation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model steady-state cost (compute, RDS, S3 storage and requests, egress) at 5,000 users and apply the obvious optimisations; set budget alarms.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost per month projected with assumptions stated; S3 lifecycle tiering applied to archive; budget alarm configured; unit cost per user reported</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-1008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Production cutover and hypercare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Execute the cutover: final data sync, DNS/route switch, agent repointed to production tools, decommission of the interim environment, and a defined hypercare period.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cutover run to a rehearsed plan with rollback available; no data loss verified by count and checksum; hypercare issues triaged daily; interim environment retired</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REG-1009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BA: production acceptance and go-live sign-off</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run acceptance against production with real users and obtain formal go-live approval.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acceptance script executed in production; defects dispositioned; signed go-live approval recorded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PM-S9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PM: sprint ceremonies, security &amp; integration coordination</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Readiness review, cutover coordination, hypercare tracking and project closure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Go/no-go held with documented decision; cutover coordinated; closure report issued</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PM-S10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PM: hypercare tracking and project closure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Final sprint PM allocation: cutover coordination, hypercare triage, closure report and handover.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hypercare issues triaged daily; closure report issued; handover acknowledged</t>
+  </si>
+  <si>
     <t xml:space="preserve">REG-701</t>
   </si>
   <si>
@@ -1022,6 +1412,15 @@
     <t xml:space="preserve">Plug the corpus into the existing agent stack: markdown projection in the agent's consumption layout, scoped MCP connectivity, chatbot guide, agent skills, citation eval.</t>
   </si>
   <si>
+    <t xml:space="preserve">Lift the local stack onto the existing AWS production platform: PostgreSQL/RDS, S3-backed corpus and markdown projection, containerised collection workers, cloud scheduling, secrets management, infrastructure-as-code, cloud-native backup/DR.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Make the read path scale: eliminate per-row object-store reads, add caching and connection pooling, horizontally scale the stateless API/UI tier, parallelise ingestion via a queue, and prove SLOs under load-test to 5,000 users.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integrate into the existing production MCP/agent platform: shared Postgres namespacing, tool registration, SSO + RBAC, per-tenant keys and quotas, observability and alerting, CI/CD and IaC, security review, cutover and hypercare.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Post-MVP: govinfo full-text connector, simple-mode overview UX, Playwright fetch, Postgres, more inventories, digests, production hardening, LLM enrichment.</t>
   </si>
   <si>
@@ -1046,7 +1445,7 @@
     <t xml:space="preserve">100%</t>
   </si>
   <si>
-    <t xml:space="preserve">Data layer, versioning, pipeline, ops</t>
+    <t xml:space="preserve">Data layer, versioning, pipeline, ops; S7-9 needs AWS/platform skills (see assumption)</t>
   </si>
   <si>
     <t xml:space="preserve">Dashboard UI, fetch layer, docs</t>
@@ -1062,6 +1461,9 @@
   </si>
   <si>
     <t xml:space="preserve">Ceremonies, RAID, reporting (non-pointed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASSUMPTION: Sprints 7-9 (AWS migration/scale) assume platform/DevOps capability — either the Backend Engineer skills up or a Platform Engineer joins. Flag as a resourcing risk if neither.</t>
   </si>
   <si>
     <t xml:space="preserve">Planned SP by sprint (dev+BA):</t>
@@ -1074,7 +1476,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1107,6 +1509,13 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="9"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1167,7 +1576,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1181,6 +1590,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1477,7 +1890,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I103"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -3317,114 +3730,114 @@
         <v>58</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
         <v>279</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="D64" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B65" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="E64" s="2" t="s">
+      <c r="C65" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="F64" s="2" t="s">
+      <c r="D65" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="G64" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="H64" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I64" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="D65" s="2" t="s">
+      <c r="E65" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="H65" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I65" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B66" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="E65" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="F65" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="G65" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="H65" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I65" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>266</v>
-      </c>
       <c r="C66" s="2" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="H66" s="2" t="n">
         <v>5</v>
       </c>
       <c r="I66" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H67" s="2" t="n">
         <v>3</v>
@@ -3433,182 +3846,1052 @@
         <v>16</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="D68" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I68" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="B69" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="E68" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="F68" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="G68" s="2" t="s">
-        <v>299</v>
-      </c>
-      <c r="H68" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I68" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>266</v>
-      </c>
       <c r="C69" s="2" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>280</v>
+        <v>303</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I69" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>280</v>
+        <v>303</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I70" s="2" t="s">
-        <v>53</v>
+        <v>16</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I71" s="2" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I72" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>266</v>
+        <v>320</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>267</v>
+        <v>321</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>280</v>
+        <v>322</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I73" s="2" t="s">
         <v>44</v>
       </c>
     </row>
+    <row r="74" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="H74" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I74" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="H75" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I75" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I76" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="H77" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I77" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="H78" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I78" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="G79" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="H79" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I79" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="F80" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="G80" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="H80" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I80" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="G81" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="H81" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I81" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="G82" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="H82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I82" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="E83" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="F83" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="G83" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="H83" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I83" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="F84" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="G84" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="H84" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I84" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="G85" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="H85" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I85" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="G86" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="H86" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I86" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="G87" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="H87" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I87" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="E88" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="F88" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="G88" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="H88" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I88" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="F89" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="G89" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="H89" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I89" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="E90" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="F90" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="G90" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="H90" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I90" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="E91" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="F91" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="G91" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="H91" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I91" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="F92" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="G92" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="H92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I92" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="E93" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="F93" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="G93" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="H93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I93" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="G94" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="H94" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I94" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="E95" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F95" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="G95" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="H95" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I95" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="F96" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="G96" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="H96" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I96" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="E97" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F97" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="G97" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="H97" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I97" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="E98" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="F98" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="G98" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="H98" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I98" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="E99" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="F99" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="G99" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="H99" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I99" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="E100" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="F100" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="G100" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="H100" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I100" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="E101" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="F101" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="G101" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="H101" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I101" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="F102" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="G102" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="H102" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I102" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="E103" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="F103" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="G103" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="H103" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I103" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I73"/>
+  <autoFilter ref="A1:I103"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3625,7 +4908,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -3638,10 +4921,10 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>320</v>
+        <v>450</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>321</v>
+        <v>451</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3652,7 +4935,7 @@
         <v>11</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>322</v>
+        <v>452</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3663,7 +4946,7 @@
         <v>61</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>323</v>
+        <v>453</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3674,7 +4957,7 @@
         <v>76</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>324</v>
+        <v>454</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3685,7 +4968,7 @@
         <v>40</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>325</v>
+        <v>455</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3696,7 +4979,7 @@
         <v>98</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>326</v>
+        <v>456</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3707,7 +4990,7 @@
         <v>165</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>327</v>
+        <v>457</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3718,7 +5001,7 @@
         <v>141</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>328</v>
+        <v>458</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3729,7 +5012,7 @@
         <v>213</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>329</v>
+        <v>459</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3740,22 +5023,55 @@
         <v>232</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>331</v>
+      <c r="C14" s="2" t="s">
+        <v>464</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C11"/>
+  <autoFilter ref="A1:C14"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3772,7 +5088,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -3785,30 +5101,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>332</v>
+        <v>465</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>333</v>
+        <v>466</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>334</v>
+        <v>467</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>335</v>
+        <v>468</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>336</v>
+        <v>469</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>338</v>
+        <v>471</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>10</v>
@@ -3817,10 +5133,10 @@
         <v>11</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>339</v>
+        <v>472</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3828,7 +5144,7 @@
         <v>33</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>338</v>
+        <v>471</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>10</v>
@@ -3837,10 +5153,10 @@
         <v>11</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>340</v>
+        <v>473</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3848,7 +5164,7 @@
         <v>44</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>338</v>
+        <v>471</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>10</v>
@@ -3857,10 +5173,10 @@
         <v>11</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>341</v>
+        <v>474</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3868,7 +5184,7 @@
         <v>53</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>342</v>
+        <v>475</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>2.5</v>
@@ -3877,10 +5193,10 @@
         <v>2</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>343</v>
+        <v>476</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3888,7 +5204,7 @@
         <v>58</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>342</v>
+        <v>475</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>2.5</v>
@@ -3897,15 +5213,20 @@
         <v>0</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>344</v>
+        <v>477</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>478</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>345</v>
+      <c r="A8" s="4" t="s">
+        <v>479</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3928,35 +5249,63 @@
         <v>233</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>280</v>
+        <v>282</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="5" t="n">
         <f aca="false">SUMIFS(Roadmap!H:H,Roadmap!D:D,"Sprint 1")</f>
         <v>31</v>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B10" s="5" t="n">
         <f aca="false">SUMIFS(Roadmap!H:H,Roadmap!D:D,"Sprint 2")</f>
         <v>36</v>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="5" t="n">
         <f aca="false">SUMIFS(Roadmap!H:H,Roadmap!D:D,"Sprint 3")</f>
         <v>36</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="5" t="n">
         <f aca="false">SUMIFS(Roadmap!H:H,Roadmap!D:D,"Sprint 4")</f>
         <v>36</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="5" t="n">
         <f aca="false">SUMIFS(Roadmap!H:H,Roadmap!D:D,"Sprint 5")</f>
         <v>33</v>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="F10" s="5" t="n">
         <f aca="false">SUMIFS(Roadmap!H:H,Roadmap!D:D,"Sprint 6")</f>
         <v>30</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="G10" s="5" t="n">
+        <f aca="false">SUMIFS(Roadmap!H:H,Roadmap!D:D,"Sprint 7")</f>
+        <v>31</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <f aca="false">SUMIFS(Roadmap!H:H,Roadmap!D:D,"Sprint 8")</f>
+        <v>33</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <f aca="false">SUMIFS(Roadmap!H:H,Roadmap!D:D,"Sprint 9")</f>
+        <v>31</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <f aca="false">SUMIFS(Roadmap!H:H,Roadmap!D:D,"Sprint 10")</f>
+        <v>36</v>
+      </c>
+      <c r="K10" s="5" t="n">
         <f aca="false">SUMIFS(Roadmap!H:H,Roadmap!D:D,"Backlog")</f>
         <v>42</v>
       </c>

</xml_diff>